<commit_message>
Import rules: resolve six open questions; clarify review counts
- tracking-code-key/v1: codes stored as trimmed, matched by an
  upper-cased key; case-only variants are one parcel, ambiguous
  spelling blocked for staff.
- scan-time-local/v1: scan times read as Asia/Phnom_Penh, source text
  kept beside the parsed UTC time.
- arrival-batch-date/v1: warning and explicit choice when the scan date
  differs from today; controlled re-review of a partly imported file.
- Names compared case-insensitively, whitespace-normalised.
- Review counts: rows vs parcels; unique = duplicates + left out +
  blocked + ready. Decisions table.
- Fixtures: s000000018 case variant; generator asserts the new counts
  and the two-days file.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test/fixtures/headers-case-and-spaces.xlsx
+++ b/test/fixtures/headers-case-and-spaces.xlsx
@@ -8,7 +8,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="134">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="136">
   <si>
     <t xml:space="preserve">scan order number</t>
   </si>
@@ -410,6 +410,12 @@
   </si>
   <si>
     <t xml:space="preserve">855123456718</t>
+  </si>
+  <si>
+    <t xml:space="preserve">s000000018</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-10 08:19:00</t>
   </si>
 </sst>
 </file>
@@ -2276,6 +2282,74 @@
         <v>39</v>
       </c>
     </row>
+    <row r="29">
+      <c r="A29" t="s" s="1">
+        <v>134</v>
+      </c>
+      <c r="B29" t="s" s="1">
+        <v>27</v>
+      </c>
+      <c r="C29" t="s" s="1">
+        <v>28</v>
+      </c>
+      <c r="D29" t="s" s="1">
+        <v>135</v>
+      </c>
+      <c r="E29" t="s" s="1">
+        <v>30</v>
+      </c>
+      <c r="F29" t="s" s="1">
+        <v>31</v>
+      </c>
+      <c r="G29" t="s" s="1">
+        <v>32</v>
+      </c>
+      <c r="H29" t="s" s="1">
+        <v>30</v>
+      </c>
+      <c r="I29" t="s" s="1">
+        <v>33</v>
+      </c>
+      <c r="J29" t="s" s="1">
+        <v>34</v>
+      </c>
+      <c r="K29" t="s" s="1">
+        <v>31</v>
+      </c>
+      <c r="L29">
+        <v>1</v>
+      </c>
+      <c r="M29">
+        <v>0.5</v>
+      </c>
+      <c r="N29">
+        <v>0.5</v>
+      </c>
+      <c r="O29">
+        <v>0</v>
+      </c>
+      <c r="P29">
+        <v>0</v>
+      </c>
+      <c r="Q29" t="s" s="1">
+        <v>35</v>
+      </c>
+      <c r="R29" t="s" s="1">
+        <v>132</v>
+      </c>
+      <c r="S29" t="s" s="1">
+        <v>133</v>
+      </c>
+      <c r="T29" t="s" s="1">
+        <v>38</v>
+      </c>
+      <c r="Y29" t="s" s="1">
+        <v>34</v>
+      </c>
+      <c r="Z29" t="s" s="1">
+        <v>39</v>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>